<commit_message>
Fix: Ajustes nos relatórios e desempenhos
</commit_message>
<xml_diff>
--- a/calendarioDinamico/backend/reports/monthly-report-69d41602c52b88b25e831e4a.xlsx
+++ b/calendarioDinamico/backend/reports/monthly-report-69d41602c52b88b25e831e4a.xlsx
@@ -565,7 +565,7 @@
         <v>9</v>
       </c>
       <c r="B10">
-        <v>230</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -581,7 +581,7 @@
         <v>11</v>
       </c>
       <c r="B12">
-        <v>90</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -629,7 +629,7 @@
         <v>17</v>
       </c>
       <c r="B18">
-        <v>0</v>
+        <v>460</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -765,7 +765,7 @@
         <v>34</v>
       </c>
       <c r="B36">
-        <v>320</v>
+        <v>460</v>
       </c>
     </row>
   </sheetData>

</xml_diff>